<commit_message>
Fix double-counted hours in the Opportunity Map
The 15 hrs/day content-creation row was an umbrella that already
contained the separately-listed video production and agent building,
pushing mapped hours to 462 against 450 actually worked. Removes the
umbrella row (the figure already lives in the hours-per-day input) and
adds an explicit unmapped-hours cell so the gap between mapped tasks
and hours actually worked is visible rather than hidden.

Verified independently: all twelve calculation cells and every task row
evaluate as intended.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8vEz3qRFKoM5pK74DPUV8
</commit_message>
<xml_diff>
--- a/outputs/casandra-opportunity-map.xlsx
+++ b/outputs/casandra-opportunity-map.xlsx
@@ -278,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -404,6 +404,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="24" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="24" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="24" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -544,22 +545,22 @@
     </comment>
     <comment ref="C6" authorId="0" shapeId="0">
       <text>
-        <t>STATED: "at least 15 hours a day trying to create content". Umbrella figure - break into sub-tasks next pass.</t>
+        <t>PARTLY BUILT: Claude Code + Higgsfield pipeline already in progress.</t>
       </text>
     </comment>
     <comment ref="C7" authorId="0" shapeId="0">
       <text>
-        <t>PARTLY BUILT: Claude Code + Higgsfield pipeline already in progress.</t>
+        <t>ESTIMATE - confirm. High cost of doing it wrong: authored IP, stays at Doing on purpose.</t>
       </text>
     </comment>
     <comment ref="C8" authorId="0" shapeId="0">
       <text>
-        <t>ESTIMATE - confirm. High cost of doing it wrong: authored IP, stays at Doing on purpose.</t>
+        <t>ESTIMATE - confirm.</t>
       </text>
     </comment>
     <comment ref="C9" authorId="0" shapeId="0">
       <text>
-        <t>ESTIMATE - confirm.</t>
+        <t>INVESTMENT, not a bleed. Listed so total hours are honest.</t>
       </text>
     </comment>
     <comment ref="C10" authorId="0" shapeId="0">
@@ -990,16 +991,16 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>Content creation (all channels, self-reported umbrella)</t>
+          <t>Social video production (TikTok / Instagram)</t>
         </is>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
-          <t>Daily</t>
+          <t>Weekly</t>
         </is>
       </c>
       <c r="E6" s="33" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="F6" s="31">
         <f>IF(D6="","",IF(D6="Daily",E6*22,IF(D6="Weekly",E6*4.33,IF(D6="Monthly",E6,IF(D6="Quarterly",E6*0.33,IF(D6="Annually",E6*0.083,""))))))</f>
@@ -1007,7 +1008,7 @@
       </c>
       <c r="G6" s="33" t="inlineStr">
         <is>
-          <t>Doing</t>
+          <t>Designing</t>
         </is>
       </c>
       <c r="H6" s="33" t="inlineStr">
@@ -1043,12 +1044,12 @@
       </c>
       <c r="B7" s="36" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Product/Delivery</t>
         </is>
       </c>
       <c r="C7" s="37" t="inlineStr">
         <is>
-          <t>Social video production (TikTok / Instagram)</t>
+          <t>Book writing</t>
         </is>
       </c>
       <c r="D7" s="38" t="inlineStr">
@@ -1057,7 +1058,7 @@
         </is>
       </c>
       <c r="E7" s="38" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F7" s="36">
         <f>IF(D7="","",IF(D7="Daily",E7*22,IF(D7="Weekly",E7*4.33,IF(D7="Monthly",E7,IF(D7="Quarterly",E7*0.33,IF(D7="Annually",E7*0.083,""))))))</f>
@@ -1065,17 +1066,17 @@
       </c>
       <c r="G7" s="38" t="inlineStr">
         <is>
-          <t>Designing</t>
+          <t>Doing</t>
         </is>
       </c>
       <c r="H7" s="38" t="inlineStr">
         <is>
-          <t>Delegating</t>
+          <t>Doing</t>
         </is>
       </c>
       <c r="I7" s="38" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J7" s="36">
@@ -1101,12 +1102,12 @@
       </c>
       <c r="B8" s="31" t="inlineStr">
         <is>
-          <t>Product/Delivery</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="C8" s="32" t="inlineStr">
         <is>
-          <t>Book writing</t>
+          <t>Agent / system building (this project)</t>
         </is>
       </c>
       <c r="D8" s="33" t="inlineStr">
@@ -1115,7 +1116,7 @@
         </is>
       </c>
       <c r="E8" s="33" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F8" s="31">
         <f>IF(D8="","",IF(D8="Daily",E8*22,IF(D8="Weekly",E8*4.33,IF(D8="Monthly",E8,IF(D8="Quarterly",E8*0.33,IF(D8="Annually",E8*0.083,""))))))</f>
@@ -1128,12 +1129,12 @@
       </c>
       <c r="H8" s="33" t="inlineStr">
         <is>
-          <t>Doing</t>
+          <t>Designing</t>
         </is>
       </c>
       <c r="I8" s="33" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J8" s="31">
@@ -1164,7 +1165,7 @@
       </c>
       <c r="C9" s="37" t="inlineStr">
         <is>
-          <t>Agent / system building (this project)</t>
+          <t>Training: speaker class, agent class, power circle</t>
         </is>
       </c>
       <c r="D9" s="38" t="inlineStr">
@@ -1173,7 +1174,7 @@
         </is>
       </c>
       <c r="E9" s="38" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F9" s="36">
         <f>IF(D9="","",IF(D9="Daily",E9*22,IF(D9="Weekly",E9*4.33,IF(D9="Monthly",E9,IF(D9="Quarterly",E9*0.33,IF(D9="Annually",E9*0.083,""))))))</f>
@@ -1186,12 +1187,12 @@
       </c>
       <c r="H9" s="38" t="inlineStr">
         <is>
-          <t>Designing</t>
+          <t>Doing</t>
         </is>
       </c>
       <c r="I9" s="38" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J9" s="36">
@@ -1212,46 +1213,18 @@
       </c>
     </row>
     <row r="10" ht="21.75" customHeight="1" s="29">
-      <c r="A10" s="31" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="31" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="C10" s="32" t="inlineStr">
-        <is>
-          <t>Training: speaker class, agent class, power circle</t>
-        </is>
-      </c>
-      <c r="D10" s="33" t="inlineStr">
-        <is>
-          <t>Weekly</t>
-        </is>
-      </c>
-      <c r="E10" s="33" t="n">
-        <v>6</v>
-      </c>
+      <c r="A10" s="31" t="n"/>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="32" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="33" t="n"/>
       <c r="F10" s="31">
         <f>IF(D10="","",IF(D10="Daily",E10*22,IF(D10="Weekly",E10*4.33,IF(D10="Monthly",E10,IF(D10="Quarterly",E10*0.33,IF(D10="Annually",E10*0.083,""))))))</f>
         <v/>
       </c>
-      <c r="G10" s="33" t="inlineStr">
-        <is>
-          <t>Doing</t>
-        </is>
-      </c>
-      <c r="H10" s="33" t="inlineStr">
-        <is>
-          <t>Doing</t>
-        </is>
-      </c>
-      <c r="I10" s="33" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
+      <c r="G10" s="33" t="n"/>
+      <c r="H10" s="33" t="n"/>
+      <c r="I10" s="33" t="n"/>
       <c r="J10" s="31">
         <f>IF(OR(F10="",I10=""),"",IF(AND(F10&gt;=8,I10&lt;&gt;"High"),"HIGH",IF(OR(F10&lt;4,I10="High"),"LOW","MEDIUM")))</f>
         <v/>
@@ -1955,11 +1928,26 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="15.75" customHeight="1" s="29"/>
+    <row r="46" ht="15.75" customHeight="1" s="29">
+      <c r="A46" s="50" t="inlineStr">
+        <is>
+          <t>HOURS NOT YET ON THIS LIST</t>
+        </is>
+      </c>
+      <c r="C46" s="53">
+        <f>C38-C44</f>
+        <v/>
+      </c>
+      <c r="D46" s="42" t="inlineStr">
+        <is>
+          <t>This is the gap between the 450 hours you work and the tasks mapped above. Breaking THIS down is the next pass - it is where the 15-hour days actually go.</t>
+        </is>
+      </c>
+    </row>
     <row r="47" ht="15.75" customHeight="1" s="29">
       <c r="A47" s="42" t="inlineStr">
         <is>
-          <t>READ THIS: "Capacity value at your rate" is what those hours WOULD bill if a client bought them. It is a ceiling, not money you lost - nobody buys 450 consulting hours a month. The number that matters is C35: at $3,500/hr you only need about 18 billable hours a month to hit $62,500. C39 shows how many hours you are working for each one of those.</t>
+          <t>READ THIS: "Capacity value at your rate" is what those hours WOULD bill if a client bought them. It is a ceiling, not money lost - nobody buys 450 consulting hours a month. The number that matters is C35: at $3,500/hr you need about 18 billable hours a month to hit $62,500. C39 shows how many hours you work for each one of those. C46 shows how many hours are still unaccounted for.</t>
         </is>
       </c>
     </row>

</xml_diff>